<commit_message>
docs: actualizar excel matriculas con conteo final
</commit_message>
<xml_diff>
--- a/data/matriculas_santa_sofia_OFICIAL.xlsx
+++ b/data/matriculas_santa_sofia_OFICIAL.xlsx
@@ -28,7 +28,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -45,6 +45,11 @@
         <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -58,10 +63,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,7 +437,6 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>BASE DE DATOS DE APARTAMENTOS Y REGISTRO DE MATRÍCULAS</t>
@@ -439,7 +444,6 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>Nota: Los coeficientes están actualizados según la Adición por Etapas de la Ley 675.</t>
@@ -447,7 +451,6 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>Bloque</t>
@@ -490,7 +493,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -533,7 +535,6 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -576,7 +577,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -619,7 +619,6 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -662,7 +661,6 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -705,7 +703,6 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -748,7 +745,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -791,7 +787,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -834,7 +829,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -877,7 +871,6 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -920,7 +913,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -963,7 +955,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1006,7 +997,6 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1049,7 +1039,6 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1092,7 +1081,6 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1135,7 +1123,6 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1178,7 +1165,6 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1221,7 +1207,6 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1264,7 +1249,6 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1307,7 +1291,6 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1350,7 +1333,6 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1393,7 +1375,6 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1436,7 +1417,6 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1479,7 +1459,6 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1522,7 +1501,6 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1565,7 +1543,6 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1608,7 +1585,6 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1651,7 +1627,6 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1694,7 +1669,6 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1737,7 +1711,6 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1780,7 +1753,6 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1823,7 +1795,6 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1866,7 +1837,6 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1909,7 +1879,6 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1952,7 +1921,6 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -1995,7 +1963,6 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2038,7 +2005,6 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2081,7 +2047,6 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2124,7 +2089,6 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2167,7 +2131,6 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2210,7 +2173,6 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2253,7 +2215,6 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2296,7 +2257,6 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr"/>
       <c r="B48" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2339,7 +2299,6 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr"/>
       <c r="B49" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2382,7 +2341,6 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr"/>
       <c r="B50" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2425,7 +2383,6 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr"/>
       <c r="B51" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2468,7 +2425,6 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr"/>
       <c r="B52" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2511,7 +2467,6 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr"/>
       <c r="B53" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2554,7 +2509,6 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr"/>
       <c r="B54" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2597,7 +2551,6 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr"/>
       <c r="B55" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2640,7 +2593,6 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr"/>
       <c r="B56" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2683,7 +2635,6 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr"/>
       <c r="B57" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2726,7 +2677,6 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr"/>
       <c r="B58" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2769,7 +2719,6 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr"/>
       <c r="B59" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2812,7 +2761,6 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr"/>
       <c r="B60" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2855,7 +2803,6 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr"/>
       <c r="B61" t="inlineStr">
         <is>
           <t>Bloque 3</t>
@@ -2898,7 +2845,6 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr"/>
       <c r="B62" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -2941,7 +2887,6 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr"/>
       <c r="B63" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -2984,7 +2929,6 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr"/>
       <c r="B64" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3027,7 +2971,6 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr"/>
       <c r="B65" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3070,7 +3013,6 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr"/>
       <c r="B66" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3113,7 +3055,6 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr"/>
       <c r="B67" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3156,7 +3097,6 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr"/>
       <c r="B68" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3199,7 +3139,6 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr"/>
       <c r="B69" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3242,7 +3181,6 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr"/>
       <c r="B70" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3285,7 +3223,6 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr"/>
       <c r="B71" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3328,7 +3265,6 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr"/>
       <c r="B72" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3371,7 +3307,6 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr"/>
       <c r="B73" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3414,7 +3349,6 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr"/>
       <c r="B74" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3457,7 +3391,6 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr"/>
       <c r="B75" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3500,7 +3433,6 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr"/>
       <c r="B76" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3543,7 +3475,6 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr"/>
       <c r="B77" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3586,7 +3517,6 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr"/>
       <c r="B78" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3629,7 +3559,6 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr"/>
       <c r="B79" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3672,7 +3601,6 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr"/>
       <c r="B80" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3715,7 +3643,6 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr"/>
       <c r="B81" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3758,7 +3685,6 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr"/>
       <c r="B82" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3801,7 +3727,6 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr"/>
       <c r="B83" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3844,7 +3769,6 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr"/>
       <c r="B84" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3887,7 +3811,6 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr"/>
       <c r="B85" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3930,7 +3853,6 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr"/>
       <c r="B86" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -3973,7 +3895,6 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr"/>
       <c r="B87" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4016,7 +3937,6 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr"/>
       <c r="B88" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4059,7 +3979,6 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr"/>
       <c r="B89" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4102,7 +4021,6 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr"/>
       <c r="B90" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4145,7 +4063,6 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr"/>
       <c r="B91" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4188,7 +4105,6 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr"/>
       <c r="B92" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4231,7 +4147,6 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr"/>
       <c r="B93" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4274,7 +4189,6 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr"/>
       <c r="B94" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4317,7 +4231,6 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr"/>
       <c r="B95" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4360,7 +4273,6 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr"/>
       <c r="B96" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4403,7 +4315,6 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr"/>
       <c r="B97" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4446,7 +4357,6 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr"/>
       <c r="B98" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4489,7 +4399,6 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr"/>
       <c r="B99" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4532,7 +4441,6 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr"/>
       <c r="B100" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4575,7 +4483,6 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr"/>
       <c r="B101" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4618,7 +4525,6 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr"/>
       <c r="B102" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4661,7 +4567,6 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" t="inlineStr"/>
       <c r="B103" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4704,7 +4609,6 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" t="inlineStr"/>
       <c r="B104" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4747,7 +4651,6 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr"/>
       <c r="B105" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4790,7 +4693,6 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" t="inlineStr"/>
       <c r="B106" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4833,7 +4735,6 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" t="inlineStr"/>
       <c r="B107" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4876,7 +4777,6 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" t="inlineStr"/>
       <c r="B108" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4919,7 +4819,6 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" t="inlineStr"/>
       <c r="B109" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -4962,7 +4861,6 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" t="inlineStr"/>
       <c r="B110" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -5005,7 +4903,6 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" t="inlineStr"/>
       <c r="B111" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -5048,7 +4945,6 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" t="inlineStr"/>
       <c r="B112" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -5091,7 +4987,6 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" t="inlineStr"/>
       <c r="B113" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -5134,7 +5029,6 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" t="inlineStr"/>
       <c r="B114" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -5177,7 +5071,6 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" t="inlineStr"/>
       <c r="B115" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -5220,7 +5113,6 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" t="inlineStr"/>
       <c r="B116" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -5263,7 +5155,6 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" t="inlineStr"/>
       <c r="B117" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -5306,7 +5197,6 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" t="inlineStr"/>
       <c r="B118" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -5349,7 +5239,6 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" t="inlineStr"/>
       <c r="B119" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -5392,7 +5281,6 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" t="inlineStr"/>
       <c r="B120" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -5435,7 +5323,6 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" t="inlineStr"/>
       <c r="B121" t="inlineStr">
         <is>
           <t>Bloque 4</t>
@@ -5478,7 +5365,6 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" t="inlineStr"/>
       <c r="B122" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -5521,7 +5407,6 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" t="inlineStr"/>
       <c r="B123" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -5564,7 +5449,6 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" t="inlineStr"/>
       <c r="B124" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -5607,7 +5491,6 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" t="inlineStr"/>
       <c r="B125" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -5650,7 +5533,6 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" t="inlineStr"/>
       <c r="B126" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -5693,7 +5575,6 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" t="inlineStr"/>
       <c r="B127" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -5736,7 +5617,6 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" t="inlineStr"/>
       <c r="B128" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -5779,7 +5659,6 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" t="inlineStr"/>
       <c r="B129" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -5822,7 +5701,6 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" t="inlineStr"/>
       <c r="B130" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -5865,7 +5743,6 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" t="inlineStr"/>
       <c r="B131" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -5908,7 +5785,6 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" t="inlineStr"/>
       <c r="B132" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -5951,7 +5827,6 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" t="inlineStr"/>
       <c r="B133" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -5994,7 +5869,6 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" t="inlineStr"/>
       <c r="B134" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6037,7 +5911,6 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" t="inlineStr"/>
       <c r="B135" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6080,7 +5953,6 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" t="inlineStr"/>
       <c r="B136" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6123,7 +5995,6 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" t="inlineStr"/>
       <c r="B137" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6166,7 +6037,6 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" t="inlineStr"/>
       <c r="B138" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6209,7 +6079,6 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" t="inlineStr"/>
       <c r="B139" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6252,7 +6121,6 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" t="inlineStr"/>
       <c r="B140" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6295,7 +6163,6 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" t="inlineStr"/>
       <c r="B141" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6338,7 +6205,6 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" t="inlineStr"/>
       <c r="B142" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6381,7 +6247,6 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" t="inlineStr"/>
       <c r="B143" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6424,7 +6289,6 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" t="inlineStr"/>
       <c r="B144" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6467,7 +6331,6 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" t="inlineStr"/>
       <c r="B145" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6510,7 +6373,6 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" t="inlineStr"/>
       <c r="B146" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6553,7 +6415,6 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" t="inlineStr"/>
       <c r="B147" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6596,7 +6457,6 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" t="inlineStr"/>
       <c r="B148" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6639,7 +6499,6 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" t="inlineStr"/>
       <c r="B149" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6682,7 +6541,6 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" t="inlineStr"/>
       <c r="B150" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6725,7 +6583,6 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" t="inlineStr"/>
       <c r="B151" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6768,7 +6625,6 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" t="inlineStr"/>
       <c r="B152" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6811,7 +6667,6 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" t="inlineStr"/>
       <c r="B153" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6854,7 +6709,6 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" t="inlineStr"/>
       <c r="B154" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6897,7 +6751,6 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" t="inlineStr"/>
       <c r="B155" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6940,7 +6793,6 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" t="inlineStr"/>
       <c r="B156" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -6983,7 +6835,6 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" t="inlineStr"/>
       <c r="B157" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7026,7 +6877,6 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" t="inlineStr"/>
       <c r="B158" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7069,7 +6919,6 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" t="inlineStr"/>
       <c r="B159" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7112,7 +6961,6 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" t="inlineStr"/>
       <c r="B160" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7155,7 +7003,6 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" t="inlineStr"/>
       <c r="B161" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7198,7 +7045,6 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" t="inlineStr"/>
       <c r="B162" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7241,7 +7087,6 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" t="inlineStr"/>
       <c r="B163" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7284,7 +7129,6 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" t="inlineStr"/>
       <c r="B164" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7327,7 +7171,6 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" t="inlineStr"/>
       <c r="B165" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7370,7 +7213,6 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" t="inlineStr"/>
       <c r="B166" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7413,7 +7255,6 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" t="inlineStr"/>
       <c r="B167" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7456,7 +7297,6 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" t="inlineStr"/>
       <c r="B168" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7499,7 +7339,6 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" t="inlineStr"/>
       <c r="B169" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7542,7 +7381,6 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" t="inlineStr"/>
       <c r="B170" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7585,7 +7423,6 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" t="inlineStr"/>
       <c r="B171" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7628,7 +7465,6 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" t="inlineStr"/>
       <c r="B172" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7671,7 +7507,6 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" t="inlineStr"/>
       <c r="B173" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7714,7 +7549,6 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" t="inlineStr"/>
       <c r="B174" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7757,7 +7591,6 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" t="inlineStr"/>
       <c r="B175" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7800,7 +7633,6 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" t="inlineStr"/>
       <c r="B176" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7843,7 +7675,6 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" t="inlineStr"/>
       <c r="B177" t="inlineStr">
         <is>
           <t>Bloque 1</t>
@@ -7886,7 +7717,6 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" t="inlineStr"/>
       <c r="B178" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -7929,7 +7759,6 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" t="inlineStr"/>
       <c r="B179" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -7972,7 +7801,6 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" t="inlineStr"/>
       <c r="B180" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8015,7 +7843,6 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" t="inlineStr"/>
       <c r="B181" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8058,7 +7885,6 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" t="inlineStr"/>
       <c r="B182" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8101,7 +7927,6 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" t="inlineStr"/>
       <c r="B183" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8144,7 +7969,6 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" t="inlineStr"/>
       <c r="B184" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8187,7 +8011,6 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" t="inlineStr"/>
       <c r="B185" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8230,7 +8053,6 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" t="inlineStr"/>
       <c r="B186" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8273,7 +8095,6 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" t="inlineStr"/>
       <c r="B187" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8316,7 +8137,6 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" t="inlineStr"/>
       <c r="B188" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8359,7 +8179,6 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" t="inlineStr"/>
       <c r="B189" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8402,7 +8221,6 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" t="inlineStr"/>
       <c r="B190" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8445,7 +8263,6 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" t="inlineStr"/>
       <c r="B191" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8488,7 +8305,6 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" t="inlineStr"/>
       <c r="B192" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8531,7 +8347,6 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" t="inlineStr"/>
       <c r="B193" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8574,7 +8389,6 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" t="inlineStr"/>
       <c r="B194" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8617,7 +8431,6 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" t="inlineStr"/>
       <c r="B195" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8660,7 +8473,6 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" t="inlineStr"/>
       <c r="B196" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8703,7 +8515,6 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" t="inlineStr"/>
       <c r="B197" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8746,7 +8557,6 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" t="inlineStr"/>
       <c r="B198" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8789,7 +8599,6 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" t="inlineStr"/>
       <c r="B199" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8832,7 +8641,6 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" t="inlineStr"/>
       <c r="B200" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8875,7 +8683,6 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" t="inlineStr"/>
       <c r="B201" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8918,7 +8725,6 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" t="inlineStr"/>
       <c r="B202" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -8961,7 +8767,6 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" t="inlineStr"/>
       <c r="B203" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9004,7 +8809,6 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" t="inlineStr"/>
       <c r="B204" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9047,7 +8851,6 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" t="inlineStr"/>
       <c r="B205" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9090,7 +8893,6 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" t="inlineStr"/>
       <c r="B206" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9133,7 +8935,6 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" t="inlineStr"/>
       <c r="B207" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9176,7 +8977,6 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" t="inlineStr"/>
       <c r="B208" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9219,7 +9019,6 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" t="inlineStr"/>
       <c r="B209" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9262,7 +9061,6 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" t="inlineStr"/>
       <c r="B210" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9305,7 +9103,6 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" t="inlineStr"/>
       <c r="B211" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9348,7 +9145,6 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" t="inlineStr"/>
       <c r="B212" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9391,7 +9187,6 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" t="inlineStr"/>
       <c r="B213" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9434,7 +9229,6 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" t="inlineStr"/>
       <c r="B214" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9477,7 +9271,6 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" t="inlineStr"/>
       <c r="B215" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9520,7 +9313,6 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" t="inlineStr"/>
       <c r="B216" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9563,7 +9355,6 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" t="inlineStr"/>
       <c r="B217" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9606,7 +9397,6 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" t="inlineStr"/>
       <c r="B218" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9649,7 +9439,6 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" t="inlineStr"/>
       <c r="B219" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9692,7 +9481,6 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" t="inlineStr"/>
       <c r="B220" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9735,7 +9523,6 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" t="inlineStr"/>
       <c r="B221" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9778,7 +9565,6 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" t="inlineStr"/>
       <c r="B222" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9821,7 +9607,6 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" t="inlineStr"/>
       <c r="B223" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9864,7 +9649,6 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" t="inlineStr"/>
       <c r="B224" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9907,7 +9691,6 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" t="inlineStr"/>
       <c r="B225" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9950,7 +9733,6 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" t="inlineStr"/>
       <c r="B226" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -9993,7 +9775,6 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" t="inlineStr"/>
       <c r="B227" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -10036,7 +9817,6 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" t="inlineStr"/>
       <c r="B228" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -10079,7 +9859,6 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" t="inlineStr"/>
       <c r="B229" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -10122,7 +9901,6 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" t="inlineStr"/>
       <c r="B230" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -10165,7 +9943,6 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" t="inlineStr"/>
       <c r="B231" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -10208,7 +9985,6 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" t="inlineStr"/>
       <c r="B232" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -10251,7 +10027,6 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" t="inlineStr"/>
       <c r="B233" t="inlineStr">
         <is>
           <t>Bloque 2</t>
@@ -10294,14 +10069,11 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" t="inlineStr"/>
       <c r="B234" t="inlineStr">
         <is>
           <t>TOTAL APARTAMENTOS (228)</t>
         </is>
       </c>
-      <c r="C234" t="inlineStr"/>
-      <c r="D234" t="inlineStr"/>
       <c r="E234" t="inlineStr">
         <is>
           <t>11,631.40</t>
@@ -10339,7 +10111,6 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>BASE DE DATOS DE PARQUEADEROS Y REGISTRO DE MATRÍCULAS</t>
@@ -10347,7 +10118,6 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>Nota: Incluye parqueaderos de carros (Sótano 1 y 2) y de motos (Fases 1 y 2).</t>
@@ -10355,7 +10125,6 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>Tipo</t>
@@ -10398,7 +10167,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -10441,7 +10209,6 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -10484,7 +10251,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -10527,7 +10293,6 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -10570,7 +10335,6 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -10613,7 +10377,6 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -10656,7 +10419,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -10699,7 +10461,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -10742,7 +10503,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -10785,7 +10545,6 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -10828,7 +10587,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -10871,7 +10629,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -10914,7 +10671,6 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -10957,7 +10713,6 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11000,7 +10755,6 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11043,7 +10797,6 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11086,7 +10839,6 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11129,7 +10881,6 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11172,7 +10923,6 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11215,7 +10965,6 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11258,7 +11007,6 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11301,7 +11049,6 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11344,7 +11091,6 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11387,7 +11133,6 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11430,7 +11175,6 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11473,7 +11217,6 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11516,7 +11259,6 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11559,7 +11301,6 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11602,7 +11343,6 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11645,7 +11385,6 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11688,7 +11427,6 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11731,7 +11469,6 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11774,7 +11511,6 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11817,7 +11553,6 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11860,7 +11595,6 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11903,7 +11637,6 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11946,7 +11679,6 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -11989,7 +11721,6 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12032,7 +11763,6 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12075,7 +11805,6 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12118,7 +11847,6 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12161,7 +11889,6 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12204,7 +11931,6 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr"/>
       <c r="B48" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12247,7 +11973,6 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr"/>
       <c r="B49" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12290,7 +12015,6 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr"/>
       <c r="B50" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12333,7 +12057,6 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr"/>
       <c r="B51" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12376,7 +12099,6 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr"/>
       <c r="B52" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12419,7 +12141,6 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr"/>
       <c r="B53" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12462,7 +12183,6 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr"/>
       <c r="B54" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12505,7 +12225,6 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr"/>
       <c r="B55" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12548,7 +12267,6 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr"/>
       <c r="B56" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12591,7 +12309,6 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr"/>
       <c r="B57" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12634,7 +12351,6 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr"/>
       <c r="B58" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12677,7 +12393,6 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr"/>
       <c r="B59" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12720,7 +12435,6 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr"/>
       <c r="B60" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12763,7 +12477,6 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr"/>
       <c r="B61" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12806,7 +12519,6 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr"/>
       <c r="B62" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12849,7 +12561,6 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr"/>
       <c r="B63" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12892,7 +12603,6 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr"/>
       <c r="B64" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12935,7 +12645,6 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr"/>
       <c r="B65" t="inlineStr">
         <is>
           <t>Carro Sótano 2</t>
@@ -12978,7 +12687,6 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr"/>
       <c r="B66" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13021,7 +12729,6 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr"/>
       <c r="B67" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13064,7 +12771,6 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr"/>
       <c r="B68" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13107,7 +12813,6 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr"/>
       <c r="B69" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13150,7 +12855,6 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr"/>
       <c r="B70" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13193,7 +12897,6 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr"/>
       <c r="B71" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13236,7 +12939,6 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr"/>
       <c r="B72" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13279,7 +12981,6 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr"/>
       <c r="B73" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13322,7 +13023,6 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr"/>
       <c r="B74" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13365,7 +13065,6 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr"/>
       <c r="B75" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13408,7 +13107,6 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr"/>
       <c r="B76" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13451,7 +13149,6 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr"/>
       <c r="B77" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13494,7 +13191,6 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr"/>
       <c r="B78" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13537,7 +13233,6 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr"/>
       <c r="B79" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13580,7 +13275,6 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr"/>
       <c r="B80" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13623,7 +13317,6 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr"/>
       <c r="B81" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13666,7 +13359,6 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr"/>
       <c r="B82" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13709,7 +13401,6 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr"/>
       <c r="B83" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13752,7 +13443,6 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr"/>
       <c r="B84" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13795,7 +13485,6 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr"/>
       <c r="B85" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13838,7 +13527,6 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr"/>
       <c r="B86" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13881,7 +13569,6 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr"/>
       <c r="B87" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13924,7 +13611,6 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr"/>
       <c r="B88" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -13967,7 +13653,6 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr"/>
       <c r="B89" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14010,7 +13695,6 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr"/>
       <c r="B90" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14053,7 +13737,6 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr"/>
       <c r="B91" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14096,7 +13779,6 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr"/>
       <c r="B92" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14139,7 +13821,6 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr"/>
       <c r="B93" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14182,7 +13863,6 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr"/>
       <c r="B94" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14225,7 +13905,6 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr"/>
       <c r="B95" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14268,7 +13947,6 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr"/>
       <c r="B96" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14311,7 +13989,6 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr"/>
       <c r="B97" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14354,7 +14031,6 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr"/>
       <c r="B98" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14397,7 +14073,6 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr"/>
       <c r="B99" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14440,7 +14115,6 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr"/>
       <c r="B100" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14483,7 +14157,6 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr"/>
       <c r="B101" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14526,7 +14199,6 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr"/>
       <c r="B102" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14569,7 +14241,6 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" t="inlineStr"/>
       <c r="B103" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14612,7 +14283,6 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" t="inlineStr"/>
       <c r="B104" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14655,7 +14325,6 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr"/>
       <c r="B105" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14698,7 +14367,6 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" t="inlineStr"/>
       <c r="B106" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14741,7 +14409,6 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" t="inlineStr"/>
       <c r="B107" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14784,7 +14451,6 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" t="inlineStr"/>
       <c r="B108" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14827,7 +14493,6 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" t="inlineStr"/>
       <c r="B109" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14870,7 +14535,6 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" t="inlineStr"/>
       <c r="B110" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14913,7 +14577,6 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" t="inlineStr"/>
       <c r="B111" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14956,7 +14619,6 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" t="inlineStr"/>
       <c r="B112" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -14999,7 +14661,6 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" t="inlineStr"/>
       <c r="B113" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -15042,7 +14703,6 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" t="inlineStr"/>
       <c r="B114" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -15085,7 +14745,6 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" t="inlineStr"/>
       <c r="B115" t="inlineStr">
         <is>
           <t>Carro Sótano 1</t>
@@ -15128,7 +14787,6 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" t="inlineStr"/>
       <c r="B116" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15171,7 +14829,6 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" t="inlineStr"/>
       <c r="B117" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15214,7 +14871,6 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" t="inlineStr"/>
       <c r="B118" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15257,7 +14913,6 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" t="inlineStr"/>
       <c r="B119" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15300,7 +14955,6 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" t="inlineStr"/>
       <c r="B120" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15343,7 +14997,6 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" t="inlineStr"/>
       <c r="B121" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15386,7 +15039,6 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" t="inlineStr"/>
       <c r="B122" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15429,7 +15081,6 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" t="inlineStr"/>
       <c r="B123" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15472,7 +15123,6 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" t="inlineStr"/>
       <c r="B124" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15515,7 +15165,6 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" t="inlineStr"/>
       <c r="B125" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15558,7 +15207,6 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" t="inlineStr"/>
       <c r="B126" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15601,7 +15249,6 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" t="inlineStr"/>
       <c r="B127" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15644,7 +15291,6 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" t="inlineStr"/>
       <c r="B128" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15687,7 +15333,6 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" t="inlineStr"/>
       <c r="B129" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15730,7 +15375,6 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" t="inlineStr"/>
       <c r="B130" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15773,7 +15417,6 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" t="inlineStr"/>
       <c r="B131" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15816,7 +15459,6 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" t="inlineStr"/>
       <c r="B132" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15859,7 +15501,6 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" t="inlineStr"/>
       <c r="B133" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15902,7 +15543,6 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" t="inlineStr"/>
       <c r="B134" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15945,7 +15585,6 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" t="inlineStr"/>
       <c r="B135" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -15988,7 +15627,6 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" t="inlineStr"/>
       <c r="B136" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16031,7 +15669,6 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" t="inlineStr"/>
       <c r="B137" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16074,7 +15711,6 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" t="inlineStr"/>
       <c r="B138" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16117,7 +15753,6 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" t="inlineStr"/>
       <c r="B139" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16160,7 +15795,6 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" t="inlineStr"/>
       <c r="B140" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16203,7 +15837,6 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" t="inlineStr"/>
       <c r="B141" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16246,7 +15879,6 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" t="inlineStr"/>
       <c r="B142" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16289,7 +15921,6 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" t="inlineStr"/>
       <c r="B143" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16332,7 +15963,6 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" t="inlineStr"/>
       <c r="B144" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16375,7 +16005,6 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" t="inlineStr"/>
       <c r="B145" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16418,7 +16047,6 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" t="inlineStr"/>
       <c r="B146" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16461,7 +16089,6 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" t="inlineStr"/>
       <c r="B147" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16504,7 +16131,6 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" t="inlineStr"/>
       <c r="B148" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16547,7 +16173,6 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" t="inlineStr"/>
       <c r="B149" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16590,7 +16215,6 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" t="inlineStr"/>
       <c r="B150" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16633,7 +16257,6 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" t="inlineStr"/>
       <c r="B151" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16676,7 +16299,6 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" t="inlineStr"/>
       <c r="B152" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16719,7 +16341,6 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" t="inlineStr"/>
       <c r="B153" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16762,7 +16383,6 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" t="inlineStr"/>
       <c r="B154" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16805,7 +16425,6 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" t="inlineStr"/>
       <c r="B155" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16848,7 +16467,6 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" t="inlineStr"/>
       <c r="B156" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16891,7 +16509,6 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" t="inlineStr"/>
       <c r="B157" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16934,7 +16551,6 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" t="inlineStr"/>
       <c r="B158" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -16977,7 +16593,6 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" t="inlineStr"/>
       <c r="B159" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17020,7 +16635,6 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" t="inlineStr"/>
       <c r="B160" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17063,7 +16677,6 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" t="inlineStr"/>
       <c r="B161" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17106,7 +16719,6 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" t="inlineStr"/>
       <c r="B162" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17149,7 +16761,6 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" t="inlineStr"/>
       <c r="B163" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17192,7 +16803,6 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" t="inlineStr"/>
       <c r="B164" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17235,7 +16845,6 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" t="inlineStr"/>
       <c r="B165" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17278,7 +16887,6 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" t="inlineStr"/>
       <c r="B166" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17321,7 +16929,6 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" t="inlineStr"/>
       <c r="B167" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17364,7 +16971,6 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" t="inlineStr"/>
       <c r="B168" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17407,7 +17013,6 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" t="inlineStr"/>
       <c r="B169" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17450,7 +17055,6 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" t="inlineStr"/>
       <c r="B170" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17493,7 +17097,6 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" t="inlineStr"/>
       <c r="B171" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17536,7 +17139,6 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" t="inlineStr"/>
       <c r="B172" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17579,7 +17181,6 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" t="inlineStr"/>
       <c r="B173" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17622,7 +17223,6 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" t="inlineStr"/>
       <c r="B174" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17665,7 +17265,6 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" t="inlineStr"/>
       <c r="B175" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17708,7 +17307,6 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" t="inlineStr"/>
       <c r="B176" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17751,7 +17349,6 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" t="inlineStr"/>
       <c r="B177" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17794,7 +17391,6 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" t="inlineStr"/>
       <c r="B178" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17837,7 +17433,6 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" t="inlineStr"/>
       <c r="B179" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17880,7 +17475,6 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" t="inlineStr"/>
       <c r="B180" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17923,7 +17517,6 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" t="inlineStr"/>
       <c r="B181" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -17966,7 +17559,6 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" t="inlineStr"/>
       <c r="B182" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18009,7 +17601,6 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" t="inlineStr"/>
       <c r="B183" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18052,7 +17643,6 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" t="inlineStr"/>
       <c r="B184" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18095,7 +17685,6 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" t="inlineStr"/>
       <c r="B185" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18138,7 +17727,6 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" t="inlineStr"/>
       <c r="B186" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18181,7 +17769,6 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" t="inlineStr"/>
       <c r="B187" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18224,7 +17811,6 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" t="inlineStr"/>
       <c r="B188" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18267,7 +17853,6 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" t="inlineStr"/>
       <c r="B189" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18310,7 +17895,6 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" t="inlineStr"/>
       <c r="B190" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18353,7 +17937,6 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" t="inlineStr"/>
       <c r="B191" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18396,7 +17979,6 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" t="inlineStr"/>
       <c r="B192" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18439,7 +18021,6 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" t="inlineStr"/>
       <c r="B193" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18482,7 +18063,6 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" t="inlineStr"/>
       <c r="B194" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18525,7 +18105,6 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" t="inlineStr"/>
       <c r="B195" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18568,7 +18147,6 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" t="inlineStr"/>
       <c r="B196" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18611,7 +18189,6 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" t="inlineStr"/>
       <c r="B197" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18654,7 +18231,6 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" t="inlineStr"/>
       <c r="B198" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18697,7 +18273,6 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" t="inlineStr"/>
       <c r="B199" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18740,7 +18315,6 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" t="inlineStr"/>
       <c r="B200" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18783,7 +18357,6 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" t="inlineStr"/>
       <c r="B201" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18826,7 +18399,6 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" t="inlineStr"/>
       <c r="B202" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18869,7 +18441,6 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" t="inlineStr"/>
       <c r="B203" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18912,7 +18483,6 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" t="inlineStr"/>
       <c r="B204" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18955,7 +18525,6 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" t="inlineStr"/>
       <c r="B205" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -18998,7 +18567,6 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" t="inlineStr"/>
       <c r="B206" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -19041,7 +18609,6 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" t="inlineStr"/>
       <c r="B207" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa I)</t>
@@ -19084,7 +18651,6 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" t="inlineStr"/>
       <c r="B208" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19127,7 +18693,6 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" t="inlineStr"/>
       <c r="B209" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19170,7 +18735,6 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" t="inlineStr"/>
       <c r="B210" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19213,7 +18777,6 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" t="inlineStr"/>
       <c r="B211" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19256,7 +18819,6 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" t="inlineStr"/>
       <c r="B212" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19299,7 +18861,6 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" t="inlineStr"/>
       <c r="B213" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19342,7 +18903,6 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" t="inlineStr"/>
       <c r="B214" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19385,7 +18945,6 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" t="inlineStr"/>
       <c r="B215" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19428,7 +18987,6 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" t="inlineStr"/>
       <c r="B216" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19471,7 +19029,6 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" t="inlineStr"/>
       <c r="B217" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19514,7 +19071,6 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" t="inlineStr"/>
       <c r="B218" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19557,7 +19113,6 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" t="inlineStr"/>
       <c r="B219" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19600,7 +19155,6 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" t="inlineStr"/>
       <c r="B220" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19643,7 +19197,6 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" t="inlineStr"/>
       <c r="B221" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19686,7 +19239,6 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" t="inlineStr"/>
       <c r="B222" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19729,7 +19281,6 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" t="inlineStr"/>
       <c r="B223" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19760,19 +19311,18 @@
           <t>0.013%</t>
         </is>
       </c>
-      <c r="H223" s="2" t="inlineStr">
+      <c r="H223" s="3" t="inlineStr">
         <is>
           <t>280-21XXXX</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
         <is>
-          <t>AMBIGUA: revisar manualmente opciones 280-226117, 280-226125</t>
+          <t>AMBIGUA: revisar 280-226117, 280-226125</t>
         </is>
       </c>
     </row>
     <row r="224">
-      <c r="A224" t="inlineStr"/>
       <c r="B224" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19815,7 +19365,6 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" t="inlineStr"/>
       <c r="B225" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19858,7 +19407,6 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" t="inlineStr"/>
       <c r="B226" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19901,7 +19449,6 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" t="inlineStr"/>
       <c r="B227" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19944,7 +19491,6 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" t="inlineStr"/>
       <c r="B228" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -19987,7 +19533,6 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" t="inlineStr"/>
       <c r="B229" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -20030,7 +19575,6 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" t="inlineStr"/>
       <c r="B230" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -20073,7 +19617,6 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" t="inlineStr"/>
       <c r="B231" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -20116,7 +19659,6 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" t="inlineStr"/>
       <c r="B232" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -20159,7 +19701,6 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" t="inlineStr"/>
       <c r="B233" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -20202,7 +19743,6 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" t="inlineStr"/>
       <c r="B234" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -20245,7 +19785,6 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" t="inlineStr"/>
       <c r="B235" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -20288,7 +19827,6 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" t="inlineStr"/>
       <c r="B236" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -20331,7 +19869,6 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" t="inlineStr"/>
       <c r="B237" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -20374,7 +19911,6 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" t="inlineStr"/>
       <c r="B238" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -20417,7 +19953,6 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" t="inlineStr"/>
       <c r="B239" t="inlineStr">
         <is>
           <t>Moto Privada (Etapa II)</t>
@@ -20460,14 +19995,11 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" t="inlineStr"/>
       <c r="B240" t="inlineStr">
         <is>
           <t>TOTAL PARQUEADEROS (234)</t>
         </is>
       </c>
-      <c r="C240" t="inlineStr"/>
-      <c r="D240" t="inlineStr"/>
       <c r="E240" t="inlineStr">
         <is>
           <t>1,287.40</t>
@@ -20505,7 +20037,6 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>SANTA SOFÍA CLUB RESIDENCIAL</t>
@@ -20513,7 +20044,6 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>SISTEMA DE CONTROL Y REGISTRO DE MATRÍCULAS INMOBILIARIAS</t>
@@ -20521,7 +20051,6 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>Generated Sep 2026 | v1.0 | Base de datos master de la copropiedad</t>
@@ -20529,7 +20058,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>RANGOS OFICIALES DE MATRÍCULAS INMOBILIARIAS (SEGÚN ESCRITURAS)</t>
@@ -20537,7 +20065,6 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
           <t>Etapa</t>
@@ -20565,7 +20092,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
           <t>Etapa I (Fase 1)</t>
@@ -20593,7 +20119,6 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>Etapa II (Fase 2)</t>
@@ -20621,7 +20146,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t>CONVENCIÓN DE COLORES PARA LA ADMINISTRACIÓN</t>
@@ -20629,7 +20153,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
           <t>Celda de Entrada (Light Blue)</t>
@@ -20642,7 +20165,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
           <t>Celda Calculada (Light Green)</t>
@@ -20655,7 +20177,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
           <t>ESTADÍSTICAS GENERALES DE UNIDADES PRIVADAS</t>
@@ -20663,7 +20184,6 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
           <t>Tipo de Unidad</t>
@@ -20691,7 +20211,6 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
           <t>Apartamentos Torre 1 (Bloques 1, 2, 3 y 4)</t>
@@ -20719,7 +20238,6 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
           <t>Parqueaderos de Carros Privados</t>
@@ -20747,7 +20265,6 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
           <t>Parqueaderos de Motos Privados</t>
@@ -20775,7 +20292,6 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
           <t>Gran Total Copropiedad</t>

</xml_diff>

<commit_message>
fix: deduplicar moto 60 (marcar como ambigua)
</commit_message>
<xml_diff>
--- a/data/matriculas_santa_sofia_OFICIAL.xlsx
+++ b/data/matriculas_santa_sofia_OFICIAL.xlsx
@@ -28,7 +28,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -38,6 +38,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -53,9 +58,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6634,7 +6640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I230"/>
+  <dimension ref="A1:I229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13055,14 +13061,14 @@
       <c r="E207" t="inlineStr"/>
       <c r="F207" t="inlineStr"/>
       <c r="G207" t="inlineStr"/>
-      <c r="H207" s="1" t="inlineStr">
-        <is>
-          <t>280-226125</t>
+      <c r="H207" s="2" t="inlineStr">
+        <is>
+          <t>280-21XXXX</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>CONFIRMADO</t>
+          <t>AMBIGUA: revisar manualmente opciones 280-226117, 280-226125</t>
         </is>
       </c>
     </row>
@@ -13292,12 +13298,12 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Moto 60</t>
+          <t>Moto 59</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>PARQUEADERO MOTO # 60 SEGUNDA ETAPA</t>
+          <t>PARQUEADERO MOTO # 59 SEGUNDA ETAPA</t>
         </is>
       </c>
       <c r="E215" t="inlineStr"/>
@@ -13305,7 +13311,7 @@
       <c r="G215" t="inlineStr"/>
       <c r="H215" s="1" t="inlineStr">
         <is>
-          <t>280-226117</t>
+          <t>280-226116</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
@@ -13323,12 +13329,12 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Moto 59</t>
+          <t>Moto 58</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>PARQUEADERO MOTO # 59 SEGUNDA ETAPA</t>
+          <t>PARQUEADERO MOTO # 58 SEGUNDA ETAPA</t>
         </is>
       </c>
       <c r="E216" t="inlineStr"/>
@@ -13336,7 +13342,7 @@
       <c r="G216" t="inlineStr"/>
       <c r="H216" s="1" t="inlineStr">
         <is>
-          <t>280-226116</t>
+          <t>280-226115</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
@@ -13354,12 +13360,12 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Moto 58</t>
+          <t>Moto 57</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>PARQUEADERO MOTO # 58 SEGUNDA ETAPA</t>
+          <t>PARQUEADERO MOTO # 57 SEGUNDA ETAPA</t>
         </is>
       </c>
       <c r="E217" t="inlineStr"/>
@@ -13367,7 +13373,7 @@
       <c r="G217" t="inlineStr"/>
       <c r="H217" s="1" t="inlineStr">
         <is>
-          <t>280-226115</t>
+          <t>280-226114</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
@@ -13385,12 +13391,12 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Moto 57</t>
+          <t>Moto 56</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>PARQUEADERO MOTO # 57 SEGUNDA ETAPA</t>
+          <t>PARQUEADERO MOTO # 56 SEGUNDA ETAPA</t>
         </is>
       </c>
       <c r="E218" t="inlineStr"/>
@@ -13398,7 +13404,7 @@
       <c r="G218" t="inlineStr"/>
       <c r="H218" s="1" t="inlineStr">
         <is>
-          <t>280-226114</t>
+          <t>280-226113</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
@@ -13416,12 +13422,12 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Moto 56</t>
+          <t>Moto 55</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>PARQUEADERO MOTO # 56 SEGUNDA ETAPA</t>
+          <t>PARQUEADERO MOTO # 55 SEGUNDA ETAPA</t>
         </is>
       </c>
       <c r="E219" t="inlineStr"/>
@@ -13429,7 +13435,7 @@
       <c r="G219" t="inlineStr"/>
       <c r="H219" s="1" t="inlineStr">
         <is>
-          <t>280-226113</t>
+          <t>280-226112</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
@@ -13447,12 +13453,12 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Moto 55</t>
+          <t>Moto 43</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>PARQUEADERO MOTO # 55 SEGUNDA ETAPA</t>
+          <t>PARQUEADERO MOTO # 43 SEGUNDA ETAPA</t>
         </is>
       </c>
       <c r="E220" t="inlineStr"/>
@@ -13460,7 +13466,7 @@
       <c r="G220" t="inlineStr"/>
       <c r="H220" s="1" t="inlineStr">
         <is>
-          <t>280-226112</t>
+          <t>280-226111</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
@@ -13478,12 +13484,12 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>Moto 43</t>
+          <t>Moto 42</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>PARQUEADERO MOTO # 43 SEGUNDA ETAPA</t>
+          <t>PARQUEADERO MOTO # 42 SEGUNDA ETAPA</t>
         </is>
       </c>
       <c r="E221" t="inlineStr"/>
@@ -13491,7 +13497,7 @@
       <c r="G221" t="inlineStr"/>
       <c r="H221" s="1" t="inlineStr">
         <is>
-          <t>280-226111</t>
+          <t>280-226110</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
@@ -13509,12 +13515,12 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>Moto 42</t>
+          <t>Moto 41</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>PARQUEADERO MOTO # 42 SEGUNDA ETAPA</t>
+          <t>PARQUEADERO MOTO # 41 SEGUNDA ETAPA</t>
         </is>
       </c>
       <c r="E222" t="inlineStr"/>
@@ -13522,7 +13528,7 @@
       <c r="G222" t="inlineStr"/>
       <c r="H222" s="1" t="inlineStr">
         <is>
-          <t>280-226110</t>
+          <t>280-226109</t>
         </is>
       </c>
       <c r="I222" t="inlineStr">
@@ -13540,12 +13546,12 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Moto 41</t>
+          <t>Moto 40</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>PARQUEADERO MOTO # 41 SEGUNDA ETAPA</t>
+          <t>PARQUEADERO MOTO # 40 SEGUNDA ETAPA</t>
         </is>
       </c>
       <c r="E223" t="inlineStr"/>
@@ -13553,7 +13559,7 @@
       <c r="G223" t="inlineStr"/>
       <c r="H223" s="1" t="inlineStr">
         <is>
-          <t>280-226109</t>
+          <t>280-226108</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
@@ -13571,12 +13577,12 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>Moto 40</t>
+          <t>Moto 39</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>PARQUEADERO MOTO # 40 SEGUNDA ETAPA</t>
+          <t>PARQUEADERO MOTO # 39 SEGUNDA ETAPA</t>
         </is>
       </c>
       <c r="E224" t="inlineStr"/>
@@ -13584,7 +13590,7 @@
       <c r="G224" t="inlineStr"/>
       <c r="H224" s="1" t="inlineStr">
         <is>
-          <t>280-226108</t>
+          <t>280-226107</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
@@ -13602,12 +13608,12 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>Moto 39</t>
+          <t>Moto 38</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>PARQUEADERO MOTO # 39 SEGUNDA ETAPA</t>
+          <t>PARQUEADERO MOTO # 38 SEGUNDA ETAPA</t>
         </is>
       </c>
       <c r="E225" t="inlineStr"/>
@@ -13615,7 +13621,7 @@
       <c r="G225" t="inlineStr"/>
       <c r="H225" s="1" t="inlineStr">
         <is>
-          <t>280-226107</t>
+          <t>280-226106</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
@@ -13633,12 +13639,12 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Moto 38</t>
+          <t>Moto 37</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>PARQUEADERO MOTO # 38 SEGUNDA ETAPA</t>
+          <t>PARQUEADERO MOTO # 37 SEGUNDA ETAPA</t>
         </is>
       </c>
       <c r="E226" t="inlineStr"/>
@@ -13646,7 +13652,7 @@
       <c r="G226" t="inlineStr"/>
       <c r="H226" s="1" t="inlineStr">
         <is>
-          <t>280-226106</t>
+          <t>280-226105</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
@@ -13664,12 +13670,12 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Moto 37</t>
+          <t>Moto 36</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>PARQUEADERO MOTO # 37 SEGUNDA ETAPA</t>
+          <t>PARQUEADERO MOTO # 36 SEGUNDA ETAPA</t>
         </is>
       </c>
       <c r="E227" t="inlineStr"/>
@@ -13677,7 +13683,7 @@
       <c r="G227" t="inlineStr"/>
       <c r="H227" s="1" t="inlineStr">
         <is>
-          <t>280-226105</t>
+          <t>280-226104</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
@@ -13695,12 +13701,12 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Moto 36</t>
+          <t>Moto 35</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>PARQUEADERO MOTO # 36 SEGUNDA ETAPA</t>
+          <t>PARQUEADERO MOTO # 35 SEGUNDA ETAPA</t>
         </is>
       </c>
       <c r="E228" t="inlineStr"/>
@@ -13708,7 +13714,7 @@
       <c r="G228" t="inlineStr"/>
       <c r="H228" s="1" t="inlineStr">
         <is>
-          <t>280-226104</t>
+          <t>280-226103</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -13726,12 +13732,12 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Moto 35</t>
+          <t>Moto 34</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>PARQUEADERO MOTO # 35 SEGUNDA ETAPA</t>
+          <t>PARQUEADERO MOTO # 34 SEGUNDA ETAPA</t>
         </is>
       </c>
       <c r="E229" t="inlineStr"/>
@@ -13739,41 +13745,10 @@
       <c r="G229" t="inlineStr"/>
       <c r="H229" s="1" t="inlineStr">
         <is>
-          <t>280-226103</t>
+          <t>280-226102</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
-        <is>
-          <t>CONFIRMADO</t>
-        </is>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" t="inlineStr"/>
-      <c r="B230" t="inlineStr">
-        <is>
-          <t>Moto Privada (Etapa I)</t>
-        </is>
-      </c>
-      <c r="C230" t="inlineStr">
-        <is>
-          <t>Moto 34</t>
-        </is>
-      </c>
-      <c r="D230" t="inlineStr">
-        <is>
-          <t>PARQUEADERO MOTO # 34 SEGUNDA ETAPA</t>
-        </is>
-      </c>
-      <c r="E230" t="inlineStr"/>
-      <c r="F230" t="inlineStr"/>
-      <c r="G230" t="inlineStr"/>
-      <c r="H230" s="1" t="inlineStr">
-        <is>
-          <t>280-226102</t>
-        </is>
-      </c>
-      <c r="I230" t="inlineStr">
         <is>
           <t>CONFIRMADO</t>
         </is>

</xml_diff>